<commit_message>
read me and data seperated
</commit_message>
<xml_diff>
--- a/normalized_confusion_matrix.xlsx
+++ b/normalized_confusion_matrix.xlsx
@@ -493,34 +493,34 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8648068669527897</v>
+        <v>0.8714285714285714</v>
       </c>
       <c r="C2" t="n">
-        <v>0.006666666666666667</v>
+        <v>0.005458515283842794</v>
       </c>
       <c r="D2" t="n">
-        <v>0.04531722054380664</v>
+        <v>0.04704704704704705</v>
       </c>
       <c r="E2" t="n">
-        <v>0.01044932079414838</v>
+        <v>0.01165254237288136</v>
       </c>
       <c r="F2" t="n">
-        <v>0.02026431718061674</v>
+        <v>0.02152466367713005</v>
       </c>
       <c r="G2" t="n">
-        <v>0.001015228426395939</v>
+        <v>0.00103950103950104</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0.006578947368421052</v>
+        <v>0.006256517205422315</v>
       </c>
       <c r="J2" t="n">
-        <v>0.07055503292568203</v>
+        <v>0.0743801652892562</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0260950605778192</v>
+        <v>0.03033175355450237</v>
       </c>
     </row>
     <row r="3">
@@ -530,34 +530,34 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0128755364806867</v>
+        <v>0.01318681318681319</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9411111111111111</v>
+        <v>0.9366812227074236</v>
       </c>
       <c r="D3" t="n">
-        <v>0.002014098690835851</v>
+        <v>0.001001001001001001</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01044932079414838</v>
+        <v>0.01059322033898305</v>
       </c>
       <c r="F3" t="n">
-        <v>0.001762114537444934</v>
+        <v>0.002690582959641256</v>
       </c>
       <c r="G3" t="n">
-        <v>0.002030456852791878</v>
+        <v>0.002079002079002079</v>
       </c>
       <c r="H3" t="n">
-        <v>0.007619047619047619</v>
+        <v>0.005708848715509039</v>
       </c>
       <c r="I3" t="n">
-        <v>0.002192982456140351</v>
+        <v>0.001042752867570386</v>
       </c>
       <c r="J3" t="n">
-        <v>0.03104421448730009</v>
+        <v>0.02938475665748393</v>
       </c>
       <c r="K3" t="n">
-        <v>0.07642124883504194</v>
+        <v>0.07109004739336493</v>
       </c>
     </row>
     <row r="4">
@@ -567,31 +567,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.03111587982832618</v>
+        <v>0.03516483516483516</v>
       </c>
       <c r="C4" t="n">
-        <v>0.002222222222222222</v>
+        <v>0.002183406113537118</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7472306143001007</v>
+        <v>0.7457457457457457</v>
       </c>
       <c r="E4" t="n">
-        <v>0.04597701149425287</v>
+        <v>0.04766949152542373</v>
       </c>
       <c r="F4" t="n">
-        <v>0.07753303964757709</v>
+        <v>0.07354260089686099</v>
       </c>
       <c r="G4" t="n">
-        <v>0.03857868020304569</v>
+        <v>0.03638253638253638</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0419047619047619</v>
+        <v>0.03996194100856328</v>
       </c>
       <c r="I4" t="n">
-        <v>0.009868421052631578</v>
+        <v>0.01042752867570386</v>
       </c>
       <c r="J4" t="n">
-        <v>0.003762935089369708</v>
+        <v>0.006427915518824609</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -604,34 +604,34 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.006437768240343348</v>
+        <v>0.008791208791208791</v>
       </c>
       <c r="C5" t="n">
-        <v>0.005555555555555556</v>
+        <v>0.004366812227074236</v>
       </c>
       <c r="D5" t="n">
-        <v>0.05941591137965761</v>
+        <v>0.05505505505505506</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6750261233019854</v>
+        <v>0.6949152542372882</v>
       </c>
       <c r="F5" t="n">
-        <v>0.04317180616740088</v>
+        <v>0.04394618834080718</v>
       </c>
       <c r="G5" t="n">
-        <v>0.132994923857868</v>
+        <v>0.1247401247401247</v>
       </c>
       <c r="H5" t="n">
-        <v>0.05333333333333334</v>
+        <v>0.05518553758325404</v>
       </c>
       <c r="I5" t="n">
-        <v>0.02412280701754386</v>
+        <v>0.02815432742440042</v>
       </c>
       <c r="J5" t="n">
-        <v>0.01411100658513641</v>
+        <v>0.01285583103764922</v>
       </c>
       <c r="K5" t="n">
-        <v>0.01025163094128611</v>
+        <v>0.008530805687203791</v>
       </c>
     </row>
     <row r="6">
@@ -641,34 +641,34 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.006437768240343348</v>
+        <v>0.006593406593406593</v>
       </c>
       <c r="C6" t="n">
-        <v>0.001111111111111111</v>
+        <v>0.001091703056768559</v>
       </c>
       <c r="D6" t="n">
-        <v>0.04632426988922457</v>
+        <v>0.04804804804804805</v>
       </c>
       <c r="E6" t="n">
-        <v>0.04179728317659352</v>
+        <v>0.03601694915254237</v>
       </c>
       <c r="F6" t="n">
-        <v>0.7127753303964758</v>
+        <v>0.7192825112107624</v>
       </c>
       <c r="G6" t="n">
-        <v>0.01725888324873097</v>
+        <v>0.01663201663201663</v>
       </c>
       <c r="H6" t="n">
-        <v>0.04476190476190476</v>
+        <v>0.04376784015223597</v>
       </c>
       <c r="I6" t="n">
-        <v>0.03179824561403509</v>
+        <v>0.04066736183524505</v>
       </c>
       <c r="J6" t="n">
-        <v>0.002822201317027281</v>
+        <v>0.005509641873278237</v>
       </c>
       <c r="K6" t="n">
-        <v>0.001863932898415657</v>
+        <v>0.001895734597156398</v>
       </c>
     </row>
     <row r="7">
@@ -678,34 +678,34 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.002145922746781116</v>
+        <v>0.002197802197802198</v>
       </c>
       <c r="C7" t="n">
-        <v>0.001111111111111111</v>
+        <v>0.001091703056768559</v>
       </c>
       <c r="D7" t="n">
-        <v>0.03021148036253777</v>
+        <v>0.03503503503503504</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1264367816091954</v>
+        <v>0.1207627118644068</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03876651982378854</v>
+        <v>0.03766816143497758</v>
       </c>
       <c r="G7" t="n">
-        <v>0.732994923857868</v>
+        <v>0.7463617463617463</v>
       </c>
       <c r="H7" t="n">
-        <v>0.03142857142857143</v>
+        <v>0.03139866793529972</v>
       </c>
       <c r="I7" t="n">
-        <v>0.04276315789473684</v>
+        <v>0.04900938477580814</v>
       </c>
       <c r="J7" t="n">
-        <v>0.004703668861712135</v>
+        <v>0.004591368227731864</v>
       </c>
       <c r="K7" t="n">
-        <v>0.002795899347623486</v>
+        <v>0.002843601895734597</v>
       </c>
     </row>
     <row r="8">
@@ -715,34 +715,34 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.004291845493562232</v>
+        <v>0.004395604395604396</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0.04128902316213495</v>
+        <v>0.03703703703703703</v>
       </c>
       <c r="E8" t="n">
-        <v>0.03970741901776385</v>
+        <v>0.03813559322033899</v>
       </c>
       <c r="F8" t="n">
-        <v>0.03348017621145374</v>
+        <v>0.03677130044843049</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0182741116751269</v>
+        <v>0.01663201663201663</v>
       </c>
       <c r="H8" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.8125594671741199</v>
       </c>
       <c r="I8" t="n">
-        <v>0.008771929824561403</v>
+        <v>0.009384775808133473</v>
       </c>
       <c r="J8" t="n">
-        <v>0.0009407337723424271</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0.001863932898415657</v>
+        <v>0.002843601895734597</v>
       </c>
     </row>
     <row r="9">
@@ -752,34 +752,34 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.01609442060085837</v>
+        <v>0.01318681318681319</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>0.001091703056768559</v>
       </c>
       <c r="D9" t="n">
-        <v>0.01409869083585096</v>
+        <v>0.01701701701701702</v>
       </c>
       <c r="E9" t="n">
-        <v>0.03657262277951933</v>
+        <v>0.02860169491525424</v>
       </c>
       <c r="F9" t="n">
-        <v>0.06343612334801763</v>
+        <v>0.05650224215246637</v>
       </c>
       <c r="G9" t="n">
-        <v>0.05482233502538071</v>
+        <v>0.05301455301455302</v>
       </c>
       <c r="H9" t="n">
-        <v>0.006666666666666667</v>
+        <v>0.007611798287345386</v>
       </c>
       <c r="I9" t="n">
-        <v>0.8673245614035088</v>
+        <v>0.8467153284671532</v>
       </c>
       <c r="J9" t="n">
-        <v>0.003762935089369708</v>
+        <v>0.003673094582185491</v>
       </c>
       <c r="K9" t="n">
-        <v>0.007455731593662628</v>
+        <v>0.004739336492890996</v>
       </c>
     </row>
     <row r="10">
@@ -789,34 +789,34 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.04506437768240344</v>
+        <v>0.03736263736263736</v>
       </c>
       <c r="C10" t="n">
-        <v>0.01111111111111111</v>
+        <v>0.01200873362445415</v>
       </c>
       <c r="D10" t="n">
-        <v>0.01007049345417925</v>
+        <v>0.01001001001001001</v>
       </c>
       <c r="E10" t="n">
-        <v>0.008359456635318705</v>
+        <v>0.006355932203389831</v>
       </c>
       <c r="F10" t="n">
-        <v>0.004405286343612335</v>
+        <v>0.004484304932735426</v>
       </c>
       <c r="G10" t="n">
-        <v>0.001015228426395939</v>
+        <v>0.002079002079002079</v>
       </c>
       <c r="H10" t="n">
-        <v>0.002857142857142857</v>
+        <v>0.00285442435775452</v>
       </c>
       <c r="I10" t="n">
-        <v>0.002192982456140351</v>
+        <v>0.003128258602711158</v>
       </c>
       <c r="J10" t="n">
-        <v>0.8494825964252116</v>
+        <v>0.8383838383838383</v>
       </c>
       <c r="K10" t="n">
-        <v>0.01491146318732526</v>
+        <v>0.01232227488151659</v>
       </c>
     </row>
     <row r="11">
@@ -826,34 +826,34 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.01072961373390558</v>
+        <v>0.007692307692307693</v>
       </c>
       <c r="C11" t="n">
-        <v>0.03111111111111111</v>
+        <v>0.03602620087336245</v>
       </c>
       <c r="D11" t="n">
-        <v>0.004028197381671702</v>
+        <v>0.004004004004004004</v>
       </c>
       <c r="E11" t="n">
-        <v>0.00522466039707419</v>
+        <v>0.005296610169491525</v>
       </c>
       <c r="F11" t="n">
-        <v>0.004405286343612335</v>
+        <v>0.003587443946188341</v>
       </c>
       <c r="G11" t="n">
-        <v>0.001015228426395939</v>
+        <v>0.00103950103950104</v>
       </c>
       <c r="H11" t="n">
-        <v>0.001904761904761905</v>
+        <v>0.0009514747859181732</v>
       </c>
       <c r="I11" t="n">
-        <v>0.004385964912280702</v>
+        <v>0.005213764337851929</v>
       </c>
       <c r="J11" t="n">
-        <v>0.01881467544684854</v>
+        <v>0.02479338842975207</v>
       </c>
       <c r="K11" t="n">
-        <v>0.8583410997204101</v>
+        <v>0.8654028436018958</v>
       </c>
     </row>
   </sheetData>

</xml_diff>